<commit_message>
kabeli NARE UNIT 1 i 2, napravljena tablica i priprema za popravke
</commit_message>
<xml_diff>
--- a/PCH_Nare/kabeli_1CJA01_2CJA01.xlsx
+++ b/PCH_Nare/kabeli_1CJA01_2CJA01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\odojak\Brodotehna\Projekti\PCH_Nare\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78FE9CEE-44F8-4A6B-A0CB-9D542874DC41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C324B755-D693-4C26-884F-31CC5282274A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DC8E694B-385C-4AD4-97DA-DB14E64DCCA3}"/>
+    <workbookView xWindow="-38520" yWindow="-2700" windowWidth="38640" windowHeight="21120" tabRatio="630" xr2:uid="{DC8E694B-385C-4AD4-97DA-DB14E64DCCA3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="104">
   <si>
     <t>Kabel</t>
   </si>
@@ -221,9 +221,6 @@
     <t>CJAW176</t>
   </si>
   <si>
-    <t>CJAW177</t>
-  </si>
-  <si>
     <t>CJAW178</t>
   </si>
   <si>
@@ -269,14 +266,98 @@
     <t>0AKA02</t>
   </si>
   <si>
-    <t>vjerojatno bum moro ponovo nacrtat jer nekaj ne valja</t>
+    <t>1BFA01</t>
+  </si>
+  <si>
+    <t>2BFA01</t>
+  </si>
+  <si>
+    <t>0BFA11</t>
+  </si>
+  <si>
+    <t>0BVB01</t>
+  </si>
+  <si>
+    <t>1MKA10</t>
+  </si>
+  <si>
+    <t>2MKA10</t>
+  </si>
+  <si>
+    <t>2MEB10</t>
+  </si>
+  <si>
+    <t>1MEB10</t>
+  </si>
+  <si>
+    <t>MEX10 GH01</t>
+  </si>
+  <si>
+    <t>0CJA01</t>
+  </si>
+  <si>
+    <t>0CHG01</t>
+  </si>
+  <si>
+    <t>0CHG01, 0AKA01</t>
+  </si>
+  <si>
+    <t>MKV10 GH01</t>
+  </si>
+  <si>
+    <t>MKA10 GH01</t>
+  </si>
+  <si>
+    <t>MKF10 GH01</t>
+  </si>
+  <si>
+    <t>1MKA10 TB4</t>
+  </si>
+  <si>
+    <t>energetski kabel, bez SH</t>
+  </si>
+  <si>
+    <t>1MKC11</t>
+  </si>
+  <si>
+    <t>2MKC11</t>
+  </si>
+  <si>
+    <t>1BAA01, 1MKA10</t>
+  </si>
+  <si>
+    <t>2BAA01, 2MKA10</t>
+  </si>
+  <si>
+    <t>0AKA04</t>
+  </si>
+  <si>
+    <t>ethernet kabel</t>
+  </si>
+  <si>
+    <t>optički kabel</t>
+  </si>
+  <si>
+    <t>FALI JEDNA ŽILA NA MB/24</t>
+  </si>
+  <si>
+    <t>5-12 na MEX10 GH01 na MC/58</t>
+  </si>
+  <si>
+    <t>Ukupno žila × presjek</t>
+  </si>
+  <si>
+    <t>12 × 17</t>
+  </si>
+  <si>
+    <t>dodan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,16 +373,46 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -313,16 +424,26 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thin">
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -333,14 +454,42 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -673,390 +822,934 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95A4773B-7BE2-483B-9873-335B9FF53F29}">
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" style="5" customWidth="1"/>
-    <col min="5" max="5" width="45.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="18.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" style="4" customWidth="1"/>
+    <col min="6" max="6" width="49" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="5">
+      <c r="E2" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="5">
+      <c r="E3" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="5">
+      <c r="E4" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="5">
+      <c r="E5" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D6" s="5">
-        <v>2</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E6" s="4">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C7" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C8" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="4">
+        <v>4</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="4">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="4">
+        <v>0</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C12" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C13" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E15" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E16" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E17" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E18" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C20" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C21" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E21" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C22" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E22" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E23" s="4">
+        <v>8</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C24" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E24" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C25" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E25" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C26" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E26" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
+      <c r="C27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E27" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B28" s="14"/>
+      <c r="C28" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C29" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E29" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C30" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E30" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C31" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E31" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C32" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E32" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E33" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E34" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B35" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E35" s="4">
+        <v>7</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E36" s="4">
+        <v>3</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C37" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E37" s="4">
+        <v>0</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C38" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E38" s="4">
+        <v>0</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C39" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E39" s="4">
+        <v>0</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E40" s="4">
+        <v>6</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
+      <c r="C41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E41" s="4">
+        <v>1</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="8" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B42" s="10"/>
+      <c r="C42" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E42" s="10">
+        <v>1</v>
+      </c>
+      <c r="F42" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="G42" s="8"/>
+    </row>
+    <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C43" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E43" s="4">
+        <v>2</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C44" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E44" s="4">
+        <v>1</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C45" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E45" s="4">
+        <v>2</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C46" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E46" s="4">
+        <v>0</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C47" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E47" s="4">
+        <v>0</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
+      <c r="C48" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E48" s="4">
+        <v>0</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B49" s="14"/>
+      <c r="C49" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E49" s="4">
+        <v>0</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C50" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E50" s="4">
+        <v>0</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C51" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E51" s="4">
+        <v>0</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="C52" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E52" s="4">
+        <v>0</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" s="1" t="s">
+      <c r="C53" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E53" s="4">
+        <v>0</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="8" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B54" s="10"/>
+      <c r="C54" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E54" s="10">
+        <v>0</v>
+      </c>
+      <c r="F54" s="8"/>
+      <c r="G54" s="8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="G55" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="G56" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="G57" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="G58" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="G59" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="G60" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="G61" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A63" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
popravljeni kabeli u NARE UNIT 1 i 2
</commit_message>
<xml_diff>
--- a/PCH_Nare/kabeli_1CJA01_2CJA01.xlsx
+++ b/PCH_Nare/kabeli_1CJA01_2CJA01.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\odojak\Brodotehna\Projekti\PCH_Nare\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C324B755-D693-4C26-884F-31CC5282274A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F03799-2829-4242-93AD-C87D32CA5DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-2700" windowWidth="38640" windowHeight="21120" tabRatio="630" xr2:uid="{DC8E694B-385C-4AD4-97DA-DB14E64DCCA3}"/>
+    <workbookView xWindow="-38520" yWindow="-4155" windowWidth="38640" windowHeight="21120" tabRatio="630" xr2:uid="{DC8E694B-385C-4AD4-97DA-DB14E64DCCA3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$67</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="119">
   <si>
     <t>Kabel</t>
   </si>
@@ -290,60 +293,24 @@
     <t>1MEB10</t>
   </si>
   <si>
-    <t>MEX10 GH01</t>
-  </si>
-  <si>
     <t>0CJA01</t>
   </si>
   <si>
     <t>0CHG01</t>
   </si>
   <si>
-    <t>0CHG01, 0AKA01</t>
-  </si>
-  <si>
-    <t>MKV10 GH01</t>
-  </si>
-  <si>
-    <t>MKA10 GH01</t>
-  </si>
-  <si>
-    <t>MKF10 GH01</t>
-  </si>
-  <si>
     <t>1MKA10 TB4</t>
   </si>
   <si>
-    <t>energetski kabel, bez SH</t>
-  </si>
-  <si>
     <t>1MKC11</t>
   </si>
   <si>
     <t>2MKC11</t>
   </si>
   <si>
-    <t>1BAA01, 1MKA10</t>
-  </si>
-  <si>
-    <t>2BAA01, 2MKA10</t>
-  </si>
-  <si>
     <t>0AKA04</t>
   </si>
   <si>
-    <t>ethernet kabel</t>
-  </si>
-  <si>
-    <t>optički kabel</t>
-  </si>
-  <si>
-    <t>FALI JEDNA ŽILA NA MB/24</t>
-  </si>
-  <si>
-    <t>5-12 na MEX10 GH01 na MC/58</t>
-  </si>
-  <si>
     <t>Ukupno žila × presjek</t>
   </si>
   <si>
@@ -351,13 +318,94 @@
   </si>
   <si>
     <t>dodan</t>
+  </si>
+  <si>
+    <t>Marin  provjerava</t>
+  </si>
+  <si>
+    <t>12 × 16</t>
+  </si>
+  <si>
+    <t>1MEX10 GH01</t>
+  </si>
+  <si>
+    <t>2MKA10 TB4</t>
+  </si>
+  <si>
+    <t>4 × 17</t>
+  </si>
+  <si>
+    <t>CJAW177</t>
+  </si>
+  <si>
+    <t>4 × 10</t>
+  </si>
+  <si>
+    <t>1BAA01</t>
+  </si>
+  <si>
+    <t>2BAA01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1MEX10 GH01 </t>
+  </si>
+  <si>
+    <t>2MEX10 GH01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1MKV10 GH01 </t>
+  </si>
+  <si>
+    <t>2MKV10 GH01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1MKA10 GH01 </t>
+  </si>
+  <si>
+    <t>2MKA10 GH01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1MKF10 GH01 </t>
+  </si>
+  <si>
+    <t>2MKF10 GH01</t>
+  </si>
+  <si>
+    <t>Komentar</t>
+  </si>
+  <si>
+    <t>CJAW131</t>
+  </si>
+  <si>
+    <t>CJAW132</t>
+  </si>
+  <si>
+    <t>CJAW133</t>
+  </si>
+  <si>
+    <t>CJAW134</t>
+  </si>
+  <si>
+    <t>0AKA03</t>
+  </si>
+  <si>
+    <t>4 × 12</t>
+  </si>
+  <si>
+    <t>2MEA10 GH02</t>
+  </si>
+  <si>
+    <t>1MEA10 GH02</t>
+  </si>
+  <si>
+    <t>ethernet</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -374,20 +422,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -396,37 +437,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -439,11 +460,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -451,45 +471,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Bad" xfId="1" builtinId="27"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -822,261 +835,302 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95A4773B-7BE2-483B-9873-335B9FF53F29}">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.77734375" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.6640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" style="4" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" style="3" customWidth="1"/>
     <col min="6" max="6" width="49" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="32.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="7" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="C1" s="12" t="s">
+    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F1" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="B2" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="B3" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="B4" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="B5" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="C5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="B6" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>73</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>1</v>
       </c>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="B7" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>73</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="B8" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>73</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <v>4</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F8" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="B9" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C9" s="2" t="s">
         <v>75</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E9" s="4">
-        <v>0</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E9" s="3">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="B10" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C10" s="2" t="s">
         <v>75</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E10" s="4">
-        <v>0</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E10" s="3">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="B11" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C11" s="2" t="s">
         <v>75</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E11" s="4">
-        <v>0</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E11" s="3">
+        <v>3</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="B12" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C12" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
+      <c r="B13" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C13" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="B14" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C14" s="2" t="s">
         <v>79</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E14" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E14" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="B15" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C15" s="2" t="s">
         <v>79</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="B16" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C16" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="3">
         <v>10</v>
       </c>
     </row>
@@ -1084,13 +1138,16 @@
       <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
+      <c r="B17" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C17" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="3">
         <v>3</v>
       </c>
     </row>
@@ -1098,13 +1155,16 @@
       <c r="A18" s="1" t="s">
         <v>28</v>
       </c>
+      <c r="B18" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C18" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1112,30 +1172,33 @@
       <c r="A19" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="B19" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C19" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E19" s="4">
-        <v>0</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>100</v>
+      <c r="E19" s="3">
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>30</v>
       </c>
+      <c r="B20" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C20" s="2" t="s">
         <v>82</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1143,13 +1206,16 @@
       <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="B21" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C21" s="2" t="s">
         <v>82</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="3">
         <v>6</v>
       </c>
     </row>
@@ -1157,13 +1223,16 @@
       <c r="A22" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="B22" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C22" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="3">
         <v>6</v>
       </c>
     </row>
@@ -1171,30 +1240,33 @@
       <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
+      <c r="B23" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C23" s="2" t="s">
-        <v>7</v>
+        <v>94</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E23" s="4">
-        <v>8</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>83</v>
+        <v>102</v>
+      </c>
+      <c r="E23" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>34</v>
       </c>
+      <c r="B24" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C24" s="2" t="s">
         <v>75</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1202,27 +1274,33 @@
       <c r="A25" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="B25" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C25" s="2" t="s">
         <v>75</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E25" s="4">
-        <v>7</v>
+      <c r="E25" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>36</v>
       </c>
+      <c r="B26" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C26" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E26" s="4">
+        <v>83</v>
+      </c>
+      <c r="E26" s="3">
         <v>10</v>
       </c>
     </row>
@@ -1230,39 +1308,50 @@
       <c r="A27" s="1" t="s">
         <v>37</v>
       </c>
+      <c r="B27" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C27" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E27" s="3">
         <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>86</v>
+      <c r="B28" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E28" s="3">
+        <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="B29" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C29" s="9" t="s">
         <v>73</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E29" s="3">
         <v>1</v>
       </c>
     </row>
@@ -1270,287 +1359,310 @@
       <c r="A30" s="1" t="s">
         <v>40</v>
       </c>
+      <c r="B30" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="C30" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E30" s="4">
+      <c r="E30" s="3">
         <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
+      <c r="A31" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="B31" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E31" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E32" s="8">
+        <v>8</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E33" s="8">
+        <v>8</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="E34" s="8">
+        <v>8</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="E35" s="8">
+        <v>8</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E36" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E37" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E38" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E39" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E40" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E41" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E42" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E43" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E44" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E45" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C46" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E31" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E32" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E33" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E34" s="4">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35" s="2" t="s">
+      <c r="D46" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="E46" s="11">
         <v>1</v>
       </c>
-      <c r="E35" s="4">
-        <v>7</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E36" s="4">
-        <v>3</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E37" s="4">
-        <v>0</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E38" s="4">
-        <v>0</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E39" s="4">
-        <v>0</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E40" s="4">
-        <v>6</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E41" s="4">
-        <v>1</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B42" s="10"/>
-      <c r="C42" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="E42" s="10">
-        <v>1</v>
-      </c>
-      <c r="F42" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="G42" s="8"/>
-    </row>
-    <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
+      <c r="F46" s="10"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E43" s="4">
-        <v>2</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E44" s="4">
-        <v>1</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E45" s="4">
-        <v>2</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E46" s="4">
-        <v>0</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
-        <v>57</v>
+      <c r="B47" s="3" t="s">
+        <v>98</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>79</v>
@@ -1558,51 +1670,50 @@
       <c r="D47" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E47" s="4">
-        <v>0</v>
-      </c>
-      <c r="G47" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E47" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>115</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E48" s="4">
-        <v>0</v>
-      </c>
-      <c r="G48" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B49" s="14"/>
-      <c r="C49" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="D49" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="E49" s="4">
-        <v>0</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+      <c r="E48" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E49" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>98</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>79</v>
@@ -1610,16 +1721,16 @@
       <c r="D50" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E50" s="4">
-        <v>0</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E50" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>98</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>79</v>
@@ -1627,129 +1738,216 @@
       <c r="D51" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E51" s="4">
-        <v>0</v>
-      </c>
-      <c r="G51" s="1" t="s">
+      <c r="E51" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E52" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E53" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E54" s="3">
+        <v>2</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A52" s="1" t="s">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E55" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E56" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="B57" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="D57" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E52" s="4">
-        <v>0</v>
-      </c>
-      <c r="G52" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A53" s="1" t="s">
+      <c r="E57" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="B58" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D53" s="2" t="s">
+      <c r="D58" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E53" s="4">
-        <v>0</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="8" t="s">
+      <c r="E58" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B54" s="10"/>
-      <c r="C54" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="D54" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="E54" s="10">
-        <v>0</v>
-      </c>
-      <c r="F54" s="8"/>
-      <c r="G54" s="8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="1" t="s">
+      <c r="B59" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D59" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="E59" s="11">
+        <v>0</v>
+      </c>
+      <c r="F59" s="10"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="G55" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
+      <c r="B60" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="G56" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A57" s="1" t="s">
+      <c r="B61" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G57" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A58" s="1" t="s">
+      <c r="B62" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="G58" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A59" s="1" t="s">
+      <c r="B63" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="G59" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A60" s="1" t="s">
+      <c r="B64" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="G60" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
+      <c r="B65" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="G61" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A62" s="1" t="s">
+      <c r="B66" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="1" t="s">
         <v>72</v>
       </c>
+      <c r="F67" s="5" t="s">
+        <v>92</v>
+      </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>